<commit_message>
feat: add Supabase client and improve body parsing
Integrate @supabase/supabase-js for backend services and implement robust request body parsing to ensure compatibility with Vercel serverless environments.
</commit_message>
<xml_diff>
--- a/data/college_records.xlsx
+++ b/data/college_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K24"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -452,19 +452,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>vsb-rec-hostel-info-mv6y3zab-1</v>
+        <v>vsb-rec-faculty-department-contacts-mv7lu8c7</v>
       </c>
       <c r="C2" t="str">
-        <v>HOSTEL_INFO</v>
+        <v>FACULTY_DEPARTMENT_CONTACTS</v>
       </c>
       <c r="D2" t="str">
-        <v>Girls Hostel Krishna Block Wi-Fi &amp; Gymnasium Access</v>
+        <v>Aiml Hod</v>
       </c>
       <c r="E2" t="str">
-        <v>Girls Hostel Krishna Block features high-speed 500 Mbps Wi-Fi, dedicated yoga hall, evening indoor badminton court, and 24/7 security surveillance with biometric entry.</v>
+        <v>Dr Malani, Ma'am, is the AI/ML department HOD</v>
       </c>
       <c r="F2" t="str">
-        <v>Warden Office</v>
+        <v>Campus Office Record</v>
       </c>
       <c r="G2" t="str">
         <v>V.S.B. Engineering College</v>
@@ -476,10 +476,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-13T17:19:12.227Z</v>
+        <v>2026-10-14T04:23:28.183Z</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-10-13T17:19:12.227Z</v>
+        <v>2026-10-14T04:57:56.199Z</v>
       </c>
     </row>
     <row r="3">
@@ -487,19 +487,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>vsb-rec-transport-info-mv6y3zab-0</v>
+        <v>vsb-rec-faculty-department-contacts-mv7ir9sk</v>
       </c>
       <c r="C3" t="str">
-        <v>TRANSPORT_INFO</v>
+        <v>FACULTY_DEPARTMENT_CONTACTS</v>
       </c>
       <c r="D3" t="str">
-        <v>Bus Route 42 - Tiruppur to VSB Campus</v>
+        <v>vice principal</v>
       </c>
       <c r="E3" t="str">
-        <v>Bus Route 42 departs Tiruppur Old Bus Stand at 6:15 AM via Kangeyam and Vellakoil, arriving at VSB Engineering College campus at 7:45 AM. Bus in-charge contact: 94425 00042.</v>
+        <v>DR Kirubashankar</v>
       </c>
       <c r="F3" t="str">
-        <v>Transport Schedule 2026</v>
+        <v>Campus Office Record</v>
       </c>
       <c r="G3" t="str">
         <v>V.S.B. Engineering College</v>
@@ -511,10 +511,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-10-13T17:19:12.227Z</v>
+        <v>2026-10-14T02:57:11.252Z</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-10-13T17:19:12.227Z</v>
+        <v>2026-10-14T05:17:33.528Z</v>
       </c>
     </row>
     <row r="4">
@@ -522,19 +522,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>vsb-rec-transport-info-mv6xzqen</v>
+        <v>vsb-rec-hostel-info-mv6y3zab-1</v>
       </c>
       <c r="C4" t="str">
-        <v>TRANSPORT_INFO</v>
+        <v>HOSTEL_INFO</v>
       </c>
       <c r="D4" t="str">
-        <v>Bus Route 25 - Erode to VSB Campus</v>
+        <v>Boys hostel</v>
       </c>
       <c r="E4" t="str">
-        <v>Bus Route 25 starts from Erode Central Bus Stand at 6:40 AM and reaches VSB campus by 7:50 AM.</v>
+        <v>There are 3 boys hostel BH-1,BH-2,BH-3 with 3 sharing ,4 sharing and 5 sharing rooms</v>
       </c>
       <c r="F4" t="str">
-        <v>Transport Notice 2026</v>
+        <v>Warden Office</v>
       </c>
       <c r="G4" t="str">
         <v>V.S.B. Engineering College</v>
@@ -546,10 +546,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-10-13T17:15:54.095Z</v>
+        <v>2026-10-13T17:19:12.227Z</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-10-13T17:15:54.095Z</v>
+        <v>2026-10-14T05:04:25.743Z</v>
       </c>
     </row>
     <row r="5">
@@ -557,19 +557,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>vsb-rec-overview-01</v>
+        <v>vsb-rec-transport-info-mv6y3zab-0</v>
       </c>
       <c r="C5" t="str">
-        <v>COLLEGE_OVERVIEW</v>
+        <v>TRANSPORT_INFO</v>
       </c>
       <c r="D5" t="str">
-        <v>Institutional Profile, History and Governance</v>
+        <v>Bus Route 42 - Tiruppur to VSB Campus</v>
       </c>
       <c r="E5" t="str">
-        <v>V.S.B. Engineering College is a self-financing, autonomous technical institution established in 2002 by the V.S.B. Educational Trust (founded in 2000 by Founder-Trustee Mr. V. S. Balsamy, B.Sc., LL.B.). The college was conferred autonomous status in 2023. It is approved by the All India Council for Technical Education (AICTE), affiliated with Anna University (Chennai), accredited by NAAC, and recognized under UGC sections 2(f) and 12(B). The institutional motto is 'HARD WORK IS THE KEY TO SUCCESS'.</v>
+        <v>Bus Route 42 departs Tiruppur Old Bus Stand at 6:15 AM via Kangeyam and Vellakoil, arriving at VSB Engineering College campus at 7:45 AM. Bus in-charge contact: 94425 00042.</v>
       </c>
       <c r="F5" t="str">
-        <v>Campus Admin</v>
+        <v>Transport Schedule 2026</v>
       </c>
       <c r="G5" t="str">
         <v>V.S.B. Engineering College</v>
@@ -581,10 +581,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-10-13T13:42:37.000Z</v>
+        <v>2026-10-13T17:19:12.227Z</v>
       </c>
       <c r="K5" t="str">
-        <v>2026-10-13T13:45:00.000Z</v>
+        <v>2026-10-13T17:19:12.227Z</v>
       </c>
     </row>
     <row r="6">
@@ -592,19 +592,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>vsb-rec-address-01</v>
+        <v>vsb-rec-transport-info-mv6xzqen</v>
       </c>
       <c r="C6" t="str">
-        <v>OFFICIAL_ADDRESS_LOCATION</v>
+        <v>TRANSPORT_INFO</v>
       </c>
       <c r="D6" t="str">
-        <v>Official Campus Address and Highway Location</v>
+        <v>Bus Route 25 - Erode to VSB Campus</v>
       </c>
       <c r="E6" t="str">
-        <v>Campus Address: V.S.B. Engineering College, NH – 67 Covai Road, Karudayampalayam Post, Karur – 639 111, Tamil Nadu, India. The institution is situated along the National Highway 67 (Coimbatore–Karur Road), providing highway transit access between Karur, Tiruchirappalli, and Coimbatore.</v>
+        <v>Bus Route 25 starts from Erode Central Bus Stand at 6:40 AM and reaches VSB campus by 7:50 AM.</v>
       </c>
       <c r="F6" t="str">
-        <v>Campus Admin</v>
+        <v>Transport Notice 2026</v>
       </c>
       <c r="G6" t="str">
         <v>V.S.B. Engineering College</v>
@@ -616,10 +616,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-10-13T13:43:40.000Z</v>
+        <v>2026-10-13T17:15:54.095Z</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-10-13T13:45:00.000Z</v>
+        <v>2026-10-13T17:15:54.095Z</v>
       </c>
     </row>
     <row r="7">
@@ -627,16 +627,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>vsb-rec-contact-01</v>
+        <v>vsb-rec-overview-01</v>
       </c>
       <c r="C7" t="str">
-        <v>CONTACT_DETAILS</v>
+        <v>COLLEGE_OVERVIEW</v>
       </c>
       <c r="D7" t="str">
-        <v>Admissions Office and General Campus Contact Channels</v>
+        <v>Institutional Profile, History and Governance</v>
       </c>
       <c r="E7" t="str">
-        <v>Official Admissions Communication: Email channels include admission@vsbec.com and admission@vsbec.org. Campus postal dispatch: NH – 67 Covai Road, Karudayampalayam Post, Karur – 639 111. Note: Individual personal telephone numbers for faculty and administration officers are not published on open web channels for privacy and security; students and applicants should communicate via the designated admission email or in-person campus reception.</v>
+        <v>V.S.B. Engineering College is a self-financing, autonomous technical institution established in 2002 by the V.S.B. Educational Trust (founded in 2000 by Founder-Trustee Mr. V. S. Balsamy, B.Sc., LL.B.). The college was conferred autonomous status in 2023. It is approved by the All India Council for Technical Education (AICTE), affiliated with Anna University (Chennai), accredited by NAAC, and recognized under UGC sections 2(f) and 12(B). The institutional motto is 'HARD WORK IS THE KEY TO SUCCESS'.</v>
       </c>
       <c r="F7" t="str">
         <v>Campus Admin</v>
@@ -651,7 +651,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-10-13T13:43:40.000Z</v>
+        <v>2026-10-13T13:42:37.000Z</v>
       </c>
       <c r="K7" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -662,16 +662,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>vsb-rec-departments-01</v>
+        <v>vsb-rec-address-01</v>
       </c>
       <c r="C8" t="str">
-        <v>DEPARTMENTS_PROGRAMMES</v>
+        <v>OFFICIAL_ADDRESS_LOCATION</v>
       </c>
       <c r="D8" t="str">
-        <v>Academic Departments and Degree Programmes Offered</v>
+        <v>Official Campus Address and Highway Location</v>
       </c>
       <c r="E8" t="str">
-        <v>Undergraduate (B.E. / B.Tech) Programmes: Artificial Intelligence and Data Science (AI &amp; DS), Artificial Intelligence and Machine Learning (AI &amp; ML), Computer Science and Engineering (CSE), Computer Science and Business System (CSBS), Computer and Communication Engineering (CCE), Information Technology (IT), Electronics and Communication Engineering (ECE), Electrical and Electronics Engineering (EEE), Mechanical Engineering (MECH), Civil Engineering, and Department of Science &amp; Humanities. Postgraduate (M.E.) Programmes: M.E. Computer Science and Engineering, M.E. Applied Electronics, and M.E. Power Systems Engineering.</v>
+        <v>Campus Address: V.S.B. Engineering College, NH – 67 Covai Road, Karudayampalayam Post, Karur – 639 111, Tamil Nadu, India. The institution is situated along the National Highway 67 (Coimbatore–Karur Road), providing highway transit access between Karur, Tiruchirappalli, and Coimbatore.</v>
       </c>
       <c r="F8" t="str">
         <v>Campus Admin</v>
@@ -686,7 +686,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-10-13T13:43:05.000Z</v>
+        <v>2026-10-13T13:43:40.000Z</v>
       </c>
       <c r="K8" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -697,22 +697,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>vsb-rec-admissions-01</v>
+        <v>vsb-rec-contact-01</v>
       </c>
       <c r="C9" t="str">
-        <v>ADMISSIONS_ELIGIBILITY</v>
+        <v>CONTACT_DETAILS</v>
       </c>
       <c r="D9" t="str">
-        <v>Admissions Eligibility and TNEA Counseling Procedures</v>
+        <v>Admissions Office and General Campus Contact Channels</v>
       </c>
       <c r="E9" t="str">
-        <v>B.E. / B.Tech admission is conducted primarily through the Tamil Nadu Engineering Admissions (TNEA) single-window counseling process administered by the Directorate of Technical Education (DOTE) / Anna University, alongside the Consortium of Self-Financing Professional Colleges quota. TNEA Institution Counseling Code: 2622. General Eligibility: Candidates must have passed Higher Secondary Examination (10+2) with Mathematics, Physics, and Chemistry, adhering to the prescribed aggregate cut-off percentages determined by government guidelines.</v>
+        <v>Official Admissions Communication: Email channels include admission@vsbec.com and admission@vsbec.org. Campus postal dispatch: NH – 67 Covai Road, Karudayampalayam Post, Karur – 639 111. Note: Individual personal telephone numbers for faculty and administration officers are not published on open web channels for privacy and security; students and applicants should communicate via the designated admission email or in-person campus reception.</v>
       </c>
       <c r="F9" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G9" t="str">
-        <v>V.S.B. Engineering College / Anna University</v>
+        <v>V.S.B. Engineering College</v>
       </c>
       <c r="H9" t="str">
         <v>VERIFIED</v>
@@ -732,22 +732,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>vsb-rec-calendar-01</v>
+        <v>vsb-rec-departments-01</v>
       </c>
       <c r="C10" t="str">
-        <v>ACADEMIC_CALENDAR</v>
+        <v>DEPARTMENTS_PROGRAMMES</v>
       </c>
       <c r="D10" t="str">
-        <v>Academic Calendar Schedules and Term Dates</v>
+        <v>Academic Departments and Degree Programmes Offered</v>
       </c>
       <c r="E10" t="str">
-        <v>Specific semester commencement dates, internal assessment testing schedules, semester examination periods, and vacation schedules are issued semester-by-semester as official circulars by the Academic Council and Dean of Academics. Detailed working day calendars for ongoing semesters are not hosted on static public pages and must be referenced directly from official noticeboards or student circulars.</v>
+        <v>Undergraduate (B.E. / B.Tech) Programmes: Artificial Intelligence and Data Science (AI &amp; DS), Artificial Intelligence and Machine Learning (AI &amp; ML), Computer Science and Engineering (CSE), Computer Science and Business System (CSBS), Computer and Communication Engineering (CCE), Information Technology (IT), Electronics and Communication Engineering (ECE), Electrical and Electronics Engineering (EEE), Mechanical Engineering (MECH), Civil Engineering, and Department of Science &amp; Humanities. Postgraduate (M.E.) Programmes: M.E. Computer Science and Engineering, M.E. Applied Electronics, and M.E. Power Systems Engineering.</v>
       </c>
       <c r="F10" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G10" t="str">
-        <v>V.S.B. Engineering College Office of Academic Affairs</v>
+        <v>V.S.B. Engineering College</v>
       </c>
       <c r="H10" t="str">
         <v>VERIFIED</v>
@@ -756,7 +756,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J10" t="str">
-        <v>2026-10-13T13:44:00.000Z</v>
+        <v>2026-10-13T13:43:05.000Z</v>
       </c>
       <c r="K10" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -767,22 +767,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>vsb-rec-exams-01</v>
+        <v>vsb-rec-admissions-01</v>
       </c>
       <c r="C11" t="str">
-        <v>EXAMINATION_INFO</v>
+        <v>ADMISSIONS_ELIGIBILITY</v>
       </c>
       <c r="D11" t="str">
-        <v>Office of Controller of Examinations (COE) and Autonomous Exam Procedures</v>
+        <v>Admissions Eligibility and TNEA Counseling Procedures</v>
       </c>
       <c r="E11" t="str">
-        <v>The Office of the Controller of Examinations was formally established in 2023 following autonomous conferment. Responsibilities include: drafting examination timetables, allocating examination halls and invigilators for Continuous Internal Assessment (CIA) tests and End Semester Examinations (ESE), processing and publishing semester results, transmitting eligible candidates' CGPA records to Anna University for degree conferral, and issuing Grade Sheets, Consolidated Marksheets, Transcripts, and CGPA-to-Percentage conversion certificates.</v>
+        <v>B.E. / B.Tech admission is conducted primarily through the Tamil Nadu Engineering Admissions (TNEA) single-window counseling process administered by the Directorate of Technical Education (DOTE) / Anna University, alongside the Consortium of Self-Financing Professional Colleges quota. TNEA Institution Counseling Code: 2622. General Eligibility: Candidates must have passed Higher Secondary Examination (10+2) with Mathematics, Physics, and Chemistry, adhering to the prescribed aggregate cut-off percentages determined by government guidelines.</v>
       </c>
       <c r="F11" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G11" t="str">
-        <v>V.S.B. Engineering College Autonomous COE</v>
+        <v>V.S.B. Engineering College / Anna University</v>
       </c>
       <c r="H11" t="str">
         <v>VERIFIED</v>
@@ -791,7 +791,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J11" t="str">
-        <v>2026-10-13T13:44:18.000Z</v>
+        <v>2026-10-13T13:43:40.000Z</v>
       </c>
       <c r="K11" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -802,22 +802,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>vsb-rec-faculty-01</v>
+        <v>vsb-rec-calendar-01</v>
       </c>
       <c r="C12" t="str">
-        <v>FACULTY_DEPARTMENT_CONTACTS</v>
+        <v>ACADEMIC_CALENDAR</v>
       </c>
       <c r="D12" t="str">
-        <v>Faculty Leadership and Department Contact Policy</v>
+        <v>Academic Calendar Schedules and Term Dates</v>
       </c>
       <c r="E12" t="str">
-        <v>Each department is led by a Professor &amp; Head of the Department (e.g., Dr. Sangeetha, HoD / Computer Science and Engineering). Specific faculty mobile numbers and home addresses are private and intentionally withheld from public digital directories. Official department academic queries should be routed through department official desks via the central campus communication office.</v>
+        <v>Specific semester commencement dates, internal assessment testing schedules, semester examination periods, and vacation schedules are issued semester-by-semester as official circulars by the Academic Council and Dean of Academics. Detailed working day calendars for ongoing semesters are not hosted on static public pages and must be referenced directly from official noticeboards or student circulars.</v>
       </c>
       <c r="F12" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G12" t="str">
-        <v>V.S.B. Engineering College</v>
+        <v>V.S.B. Engineering College Office of Academic Affairs</v>
       </c>
       <c r="H12" t="str">
         <v>VERIFIED</v>
@@ -826,7 +826,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-10-13T13:44:18.000Z</v>
+        <v>2026-10-13T13:44:00.000Z</v>
       </c>
       <c r="K12" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -837,22 +837,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>vsb-rec-facilities-01</v>
+        <v>vsb-rec-exams-01</v>
       </c>
       <c r="C13" t="str">
-        <v>CAMPUS_FACILITIES</v>
+        <v>EXAMINATION_INFO</v>
       </c>
       <c r="D13" t="str">
-        <v>Campus Infrastructure, Utilities, RO Water and Amenities</v>
+        <v>Office of Controller of Examinations (COE) and Autonomous Exam Procedures</v>
       </c>
       <c r="E13" t="str">
-        <v>The campus infrastructure includes modern lecture halls, smart classrooms with multimedia facilities, dedicated laboratories for each engineering department, a mineral water plant with reverse osmosis (RO) purification supplying drinking and cooking water campus-wide, automated teller machine (ATM) services, cafeteria, medical insurance support, IP-based video surveillance, and backup generator power systems.</v>
+        <v>The Office of the Controller of Examinations was formally established in 2023 following autonomous conferment. Responsibilities include: drafting examination timetables, allocating examination halls and invigilators for Continuous Internal Assessment (CIA) tests and End Semester Examinations (ESE), processing and publishing semester results, transmitting eligible candidates' CGPA records to Anna University for degree conferral, and issuing Grade Sheets, Consolidated Marksheets, Transcripts, and CGPA-to-Percentage conversion certificates.</v>
       </c>
       <c r="F13" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G13" t="str">
-        <v>V.S.B. Engineering College</v>
+        <v>V.S.B. Engineering College Autonomous COE</v>
       </c>
       <c r="H13" t="str">
         <v>VERIFIED</v>
@@ -861,7 +861,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-10-13T13:44:08.000Z</v>
+        <v>2026-10-13T13:44:18.000Z</v>
       </c>
       <c r="K13" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -872,22 +872,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>vsb-rec-library-01</v>
+        <v>vsb-rec-faculty-01</v>
       </c>
       <c r="C14" t="str">
-        <v>LIBRARY_FACILITIES</v>
+        <v>FACULTY_DEPARTMENT_CONTACTS</v>
       </c>
       <c r="D14" t="str">
-        <v>Central Library Collections, Digital Resources and Working Hours</v>
+        <v>Faculty Leadership and Department Contact Policy</v>
       </c>
       <c r="E14" t="str">
-        <v>Established in 2002, the V.S.B. Central Library houses approximately 43,565 book volumes across engineering, technology, and management. It subscribes to 96 national and 96 international journals, alongside audio/visual media and question banks. A dedicated Digital Library with 20 workstations provides access to e-resources via the Anna University E-Resource Consortium (AUERC) and Dolphin OPAC. Working Hours: Monday to Saturday from 8:30 a.m. to 7:00 p.m.; Holidays from 8:30 a.m. to 1:00 p.m. Circulation/Transaction Timings (Book issue/return): 8:30 a.m. to 6:00 p.m.</v>
+        <v>Each department is led by a Professor &amp; Head of the Department (e.g., Dr. Sangeetha, HoD / Computer Science and Engineering). Specific faculty mobile numbers and home addresses are private and intentionally withheld from public digital directories. Official department academic queries should be routed through department official desks via the central campus communication office.</v>
       </c>
       <c r="F14" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G14" t="str">
-        <v>V.S.B. Central Library</v>
+        <v>V.S.B. Engineering College</v>
       </c>
       <c r="H14" t="str">
         <v>VERIFIED</v>
@@ -896,7 +896,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J14" t="str">
-        <v>2026-10-13T13:44:08.000Z</v>
+        <v>2026-10-13T13:44:18.000Z</v>
       </c>
       <c r="K14" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -907,22 +907,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>vsb-rec-hostel-01</v>
+        <v>vsb-rec-facilities-01</v>
       </c>
       <c r="C15" t="str">
-        <v>HOSTEL_INFO</v>
+        <v>CAMPUS_FACILITIES</v>
       </c>
       <c r="D15" t="str">
-        <v>Residential Hostels for Men and Women</v>
+        <v>Campus Infrastructure, Utilities, RO Water and Amenities</v>
       </c>
       <c r="E15" t="str">
-        <v>The college maintains separate residential hostel blocks for male and female students. Hostel amenities include clean student rooms, recreation halls, multi-gym fitness facilities, indoor sports spaces, Wi-Fi connectivity, telephone provisions, weekend film screening, and dedicated drinking water supply from the campus mineral water RO plant.</v>
+        <v>The campus infrastructure includes modern lecture halls, smart classrooms with multimedia facilities, dedicated laboratories for each engineering department, a mineral water plant with reverse osmosis (RO) purification supplying drinking and cooking water campus-wide, automated teller machine (ATM) services, cafeteria, medical insurance support, IP-based video surveillance, and backup generator power systems.</v>
       </c>
       <c r="F15" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G15" t="str">
-        <v>V.S.B. Engineering College Hostel Administration</v>
+        <v>V.S.B. Engineering College</v>
       </c>
       <c r="H15" t="str">
         <v>VERIFIED</v>
@@ -942,22 +942,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>vsb-rec-transport-01</v>
+        <v>vsb-rec-library-01</v>
       </c>
       <c r="C16" t="str">
-        <v>TRANSPORT_INFO</v>
+        <v>LIBRARY_FACILITIES</v>
       </c>
       <c r="D16" t="str">
-        <v>College Bus Transit Routes and Coverage Network</v>
+        <v>Central Library Collections, Digital Resources and Working Hours</v>
       </c>
       <c r="E16" t="str">
-        <v>V.S.B. Engineering College operates a fleet of institutional buses catering to day-scholar students and faculty across Karur district and neighbouring taluks. Documented route pickup sectors include: Pandamangalam, Pothanur, Vennamalai, S.P. Colony, Vengamedu, Aravakuruchi, Velayuthampalayam, Manmangalam, Pallapatty, Thaneerpanthal, Velur Bus Stand, P.Velur, TNPL, Kangayam, Veerasolapuram, and Vellakovil.</v>
+        <v>Established in 2002, the V.S.B. Central Library houses approximately 43,565 book volumes across engineering, technology, and management. It subscribes to 96 national and 96 international journals, alongside audio/visual media and question banks. A dedicated Digital Library with 20 workstations provides access to e-resources via the Anna University E-Resource Consortium (AUERC) and Dolphin OPAC. Working Hours: Monday to Saturday from 8:30 a.m. to 7:00 p.m.; Holidays from 8:30 a.m. to 1:00 p.m. Circulation/Transaction Timings (Book issue/return): 8:30 a.m. to 6:00 p.m.</v>
       </c>
       <c r="F16" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G16" t="str">
-        <v>V.S.B. Engineering College Transport Department</v>
+        <v>V.S.B. Central Library</v>
       </c>
       <c r="H16" t="str">
         <v>VERIFIED</v>
@@ -977,22 +977,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>vsb-rec-scholarships-01</v>
+        <v>vsb-rec-hostel-01</v>
       </c>
       <c r="C17" t="str">
-        <v>SCHOLARSHIPS_FINANCIAL_AID</v>
+        <v>HOSTEL_INFO</v>
       </c>
       <c r="D17" t="str">
-        <v>Government Scholarships and Financial Assistance Facilitation</v>
+        <v>Facility</v>
       </c>
       <c r="E17" t="str">
-        <v>Eligible enrolled students are guided through statutory government welfare schemes, including Tamil Nadu Government Post-Matric Scholarships for BC/MBC/DNC and SC/ST/SCA students, First Graduate Tuition Fee Concession, 7.5% Government School Student Quota benefits, and Central AICTE Pragati &amp; Saksham scholarship schemes. Official college scholarship circulars and annual disbursement reports are processed through the campus administrative scholarship counter.</v>
+        <v>Hostel is provided with wifi facility and washing machines</v>
       </c>
       <c r="F17" t="str">
-        <v>Campus Admin</v>
+        <v>Facilities</v>
       </c>
       <c r="G17" t="str">
-        <v>V.S.B. Engineering College Student Welfare Desk / DOTE Tamil Nadu</v>
+        <v>V.S.B. Engineering College Hostel Administration</v>
       </c>
       <c r="H17" t="str">
         <v>VERIFIED</v>
@@ -1001,10 +1001,10 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J17" t="str">
-        <v>2026-10-13T13:44:00.000Z</v>
+        <v>2026-10-13T13:44:08.000Z</v>
       </c>
       <c r="K17" t="str">
-        <v>2026-10-13T13:45:00.000Z</v>
+        <v>2026-10-14T05:08:13.087Z</v>
       </c>
     </row>
     <row r="18">
@@ -1012,22 +1012,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>vsb-rec-placement-01</v>
+        <v>vsb-rec-transport-01</v>
       </c>
       <c r="C18" t="str">
-        <v>PLACEMENT_CAREER_SERVICES</v>
+        <v>TRANSPORT_INFO</v>
       </c>
       <c r="D18" t="str">
-        <v>Training &amp; Placement Cell and Corporate Recruitment Record</v>
+        <v>College Bus Transit Routes and Coverage Network</v>
       </c>
       <c r="E18" t="str">
-        <v>The Training &amp; Placement Cell organizes regular campus interview drives, technical workshops, coding bootcamps, and soft-skill corporate readiness training. In recent placement cycles, graduating cohorts secured over 1,177 employment offers. Leading recruiters visiting the campus include TCS (186 offers across multiple salary bands), Capgemini (165 offers), UST Global (94 offers), HCL (135 offers), Mphasis (72 offers), LTM (62 offers), ITC (52 offers), Infosys (32 offers), Cognizant (30 offers), Hexaware (28 offers), Avasoft, Kaar Technologies, and product-based companies offering top packages up to 40 Lakhs.</v>
+        <v>V.S.B. Engineering College operates a fleet of institutional buses catering to day-scholar students and faculty across Karur district and neighbouring taluks. Documented route pickup sectors include: Pandamangalam, Pothanur, Vennamalai, S.P. Colony, Vengamedu, Aravakuruchi, Velayuthampalayam, Manmangalam, Pallapatty, Thaneerpanthal, Velur Bus Stand, P.Velur, TNPL, Kangayam, Veerasolapuram, and Vellakovil.</v>
       </c>
       <c r="F18" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G18" t="str">
-        <v>V.S.B. Engineering College Placement Cell</v>
+        <v>V.S.B. Engineering College Transport Department</v>
       </c>
       <c r="H18" t="str">
         <v>VERIFIED</v>
@@ -1036,7 +1036,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J18" t="str">
-        <v>2026-10-13T13:43:28.000Z</v>
+        <v>2026-10-13T13:44:08.000Z</v>
       </c>
       <c r="K18" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -1047,22 +1047,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>vsb-rec-clubs-01</v>
+        <v>vsb-rec-scholarships-01</v>
       </c>
       <c r="C19" t="str">
-        <v>STUDENT_ACTIVITIES_CLUBS</v>
+        <v>SCHOLARSHIPS_FINANCIAL_AID</v>
       </c>
       <c r="D19" t="str">
-        <v>Student Co-curricular Clubs, Technical Societies and Cultural Bodies</v>
+        <v>Government Scholarships and Financial Assistance Facilitation</v>
       </c>
       <c r="E19" t="str">
-        <v>The college fosters student skill development through diverse active clubs: Coding Club (hands-on programming challenges, open-source projects, and hackathons), Robotics Club, Electronics Club, Electrical Club, Cultural Club &amp; Fine Arts Club (music, fine arts, drama, dance), Literature Club, Eco Club, Puzzle Club, Photography Club, Entrepreneurship Development Cell (EDC), and Youth Red Cross (YRC).</v>
+        <v>Eligible enrolled students are guided through statutory government welfare schemes, including Tamil Nadu Government Post-Matric Scholarships for BC/MBC/DNC and SC/ST/SCA students, First Graduate Tuition Fee Concession, 7.5% Government School Student Quota benefits, and Central AICTE Pragati &amp; Saksham scholarship schemes. Official college scholarship circulars and annual disbursement reports are processed through the campus administrative scholarship counter.</v>
       </c>
       <c r="F19" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G19" t="str">
-        <v>V.S.B. Engineering College Student Affairs</v>
+        <v>V.S.B. Engineering College Student Welfare Desk / DOTE Tamil Nadu</v>
       </c>
       <c r="H19" t="str">
         <v>VERIFIED</v>
@@ -1071,7 +1071,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J19" t="str">
-        <v>2026-10-13T13:44:18.000Z</v>
+        <v>2026-10-13T13:44:00.000Z</v>
       </c>
       <c r="K19" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -1082,22 +1082,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>vsb-rec-policies-01</v>
+        <v>vsb-rec-placement-01</v>
       </c>
       <c r="C20" t="str">
-        <v>REGULATIONS_POLICIES</v>
+        <v>PLACEMENT_CAREER_SERVICES</v>
       </c>
       <c r="D20" t="str">
-        <v>Student Regulations, Anti-Ragging Mandate and Grievance Committees</v>
+        <v>Training &amp; Placement Cell and Corporate Recruitment Record</v>
       </c>
       <c r="E20" t="str">
-        <v>The institution maintains strict statutory committees in compliance with AICTE, Anna University, and Supreme Court directives: 1. Anti-Ragging Committee and Squad enforcing a zero-tolerance policy against any form of harassment. 2. Grievance Redressal Committee providing structured dispute and complaint redressal. 3. Internal Complaints Committee (ICC) ensuring a safe working and learning environment. Students are required to uphold academic integrity, institutional dress code, and mandatory attendance thresholds as prescribed under Anna University autonomous regulations.</v>
+        <v>The Training &amp; Placement Cell organizes regular campus interview drives, technical workshops, coding bootcamps, and soft-skill corporate readiness training. In recent placement cycles, graduating cohorts secured over 1,177 employment offers. Leading recruiters visiting the campus include TCS (186 offers across multiple salary bands), Capgemini (165 offers), UST Global (94 offers), HCL (135 offers), Mphasis (72 offers), LTM (62 offers), ITC (52 offers), Infosys (32 offers), Cognizant (30 offers), Hexaware (28 offers), Avasoft, Kaar Technologies, and product-based companies offering top packages up to 40 Lakhs.</v>
       </c>
       <c r="F20" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G20" t="str">
-        <v>V.S.B. Engineering College / AICTE</v>
+        <v>V.S.B. Engineering College Placement Cell</v>
       </c>
       <c r="H20" t="str">
         <v>VERIFIED</v>
@@ -1106,7 +1106,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J20" t="str">
-        <v>2026-10-13T13:44:18.000Z</v>
+        <v>2026-10-13T13:43:28.000Z</v>
       </c>
       <c r="K20" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -1117,22 +1117,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>vsb-rec-notices-01</v>
+        <v>vsb-rec-clubs-01</v>
       </c>
       <c r="C21" t="str">
-        <v>OFFICIAL_NOTICES</v>
+        <v>STUDENT_ACTIVITIES_CLUBS</v>
       </c>
       <c r="D21" t="str">
-        <v>Official Institutional Announcements and Circulars</v>
+        <v>Student Co-curricular Clubs, Technical Societies and Cultural Bodies</v>
       </c>
       <c r="E21" t="str">
-        <v>Official notices regarding examination timetables, seminar registrations, campus recruitment drives, IQAC composition reports, and AICTE mandatory disclosures are published on the announcements section of the official website and on internal departmental display boards.</v>
+        <v>The college fosters student skill development through diverse active clubs: Coding Club (hands-on programming challenges, open-source projects, and hackathons), Robotics Club, Electronics Club, Electrical Club, Cultural Club &amp; Fine Arts Club (music, fine arts, drama, dance), Literature Club, Eco Club, Puzzle Club, Photography Club, Entrepreneurship Development Cell (EDC), and Youth Red Cross (YRC).</v>
       </c>
       <c r="F21" t="str">
         <v>Campus Admin</v>
       </c>
       <c r="G21" t="str">
-        <v>V.S.B. Engineering College</v>
+        <v>V.S.B. Engineering College Student Affairs</v>
       </c>
       <c r="H21" t="str">
         <v>VERIFIED</v>
@@ -1141,7 +1141,7 @@
         <v>PUBLISHED</v>
       </c>
       <c r="J21" t="str">
-        <v>2026-10-13T13:43:05.000Z</v>
+        <v>2026-10-13T13:44:18.000Z</v>
       </c>
       <c r="K21" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
@@ -1152,39 +1152,109 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
+        <v>vsb-rec-policies-01</v>
+      </c>
+      <c r="C22" t="str">
+        <v>REGULATIONS_POLICIES</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Student Regulations, Anti-Ragging Mandate and Grievance Committees</v>
+      </c>
+      <c r="E22" t="str">
+        <v>The institution maintains strict statutory committees in compliance with AICTE, Anna University, and Supreme Court directives: 1. Anti-Ragging Committee and Squad enforcing a zero-tolerance policy against any form of harassment. 2. Grievance Redressal Committee providing structured dispute and complaint redressal. 3. Internal Complaints Committee (ICC) ensuring a safe working and learning environment. Students are required to uphold academic integrity, institutional dress code, and mandatory attendance thresholds as prescribed under Anna University autonomous regulations.</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Campus Admin</v>
+      </c>
+      <c r="G22" t="str">
+        <v>V.S.B. Engineering College / AICTE</v>
+      </c>
+      <c r="H22" t="str">
+        <v>VERIFIED</v>
+      </c>
+      <c r="I22" t="str">
+        <v>PUBLISHED</v>
+      </c>
+      <c r="J22" t="str">
+        <v>2026-10-13T13:44:18.000Z</v>
+      </c>
+      <c r="K22" t="str">
+        <v>2026-10-13T13:45:00.000Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>vsb-rec-notices-01</v>
+      </c>
+      <c r="C23" t="str">
+        <v>OFFICIAL_NOTICES</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Official Institutional Announcements and Circulars</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Official notices regarding examination timetables, seminar registrations, campus recruitment drives, IQAC composition reports, and AICTE mandatory disclosures are published on the announcements section of the official website and on internal departmental display boards.</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Campus Admin</v>
+      </c>
+      <c r="G23" t="str">
+        <v>V.S.B. Engineering College</v>
+      </c>
+      <c r="H23" t="str">
+        <v>VERIFIED</v>
+      </c>
+      <c r="I23" t="str">
+        <v>PUBLISHED</v>
+      </c>
+      <c r="J23" t="str">
+        <v>2026-10-13T13:43:05.000Z</v>
+      </c>
+      <c r="K23" t="str">
+        <v>2026-10-13T13:45:00.000Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
         <v>vsb-rec-faq-01</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C24" t="str">
         <v>FREQUENTLY_ASKED_QUESTIONS</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D24" t="str">
         <v>Frequently Asked Student and Applicant Questions</v>
       </c>
-      <c r="E22" t="str">
+      <c r="E24" t="str">
         <v>Common queries verified from institutional communication channels: 1. Location: NH-67, Covai Road, Karudayampalayam, Karur, Tamil Nadu. 2. Affiliation: Affiliated to Anna University, Chennai; autonomous since 2023. 3. Counseling Code: TNEA Code 2622. 4. Hostels: Separate residential hostels with Wi-Fi and RO water for boys and girls. 5. Admissions Enquiry: admission@vsbec.com / admission@vsbec.org.</v>
       </c>
-      <c r="F22" t="str">
-        <v>Campus Admin</v>
-      </c>
-      <c r="G22" t="str">
+      <c r="F24" t="str">
+        <v>Campus Admin</v>
+      </c>
+      <c r="G24" t="str">
         <v>V.S.B. Engineering College Admissions Information Desk</v>
       </c>
-      <c r="H22" t="str">
-        <v>VERIFIED</v>
-      </c>
-      <c r="I22" t="str">
-        <v>PUBLISHED</v>
-      </c>
-      <c r="J22" t="str">
+      <c r="H24" t="str">
+        <v>VERIFIED</v>
+      </c>
+      <c r="I24" t="str">
+        <v>PUBLISHED</v>
+      </c>
+      <c r="J24" t="str">
         <v>2026-10-13T13:43:40.000Z</v>
       </c>
-      <c r="K22" t="str">
+      <c r="K24" t="str">
         <v>2026-10-13T13:45:00.000Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>